<commit_message>
sistema ya funcional primera version
</commit_message>
<xml_diff>
--- a/service/resultado_consulta.xlsx
+++ b/service/resultado_consulta.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -588,7 +588,7 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
@@ -628,7 +628,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -662,7 +662,7 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
@@ -702,7 +702,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -736,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R4" t="n">
         <v>1</v>
@@ -776,7 +776,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -810,7 +810,7 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5" t="n">
         <v>1</v>
@@ -850,7 +850,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -884,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" t="n">
         <v>1</v>
@@ -924,7 +924,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -958,7 +958,7 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" t="n">
         <v>1</v>
@@ -998,7 +998,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1032,7 +1032,7 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R8" t="n">
         <v>1</v>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1106,7 +1106,7 @@
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" t="n">
         <v>1</v>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1180,7 +1180,7 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" t="n">
         <v>1</v>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1254,7 +1254,7 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1328,7 +1328,7 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" t="n">
         <v>1</v>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1402,7 +1402,7 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R13" t="n">
         <v>1</v>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1476,7 +1476,7 @@
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
         <v>1</v>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1550,7 +1550,7 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R15" t="n">
         <v>1</v>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1624,7 +1624,7 @@
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R16" t="n">
         <v>1</v>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1698,7 +1698,7 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R17" t="n">
         <v>1</v>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1772,7 +1772,7 @@
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R18" t="n">
         <v>1</v>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1846,7 +1846,7 @@
         <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R19" t="n">
         <v>1</v>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1920,7 +1920,7 @@
         <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" t="n">
         <v>1</v>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1994,7 +1994,7 @@
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R21" t="n">
         <v>1</v>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2068,7 +2068,7 @@
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R22" t="n">
         <v>1</v>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2142,7 +2142,7 @@
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R23" t="n">
         <v>1</v>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2216,7 +2216,7 @@
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R24" t="n">
         <v>1</v>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPONSABILIDAD LIMITADA</t>
+          <t>CORPORACION DE TRANSPORTE AMERICA LIMPHAR EXPRESS SOCIEDAD COMERCIAL DE RESPOSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2290,7 +2290,7 @@
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R25" t="n">
         <v>1</v>
@@ -2364,7 +2364,7 @@
         <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R26" t="n">
         <v>1</v>
@@ -2438,7 +2438,7 @@
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R27" t="n">
         <v>1</v>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>La Factura Electrónica E001-678 no existe en los registros de SUNAT.</t>
+          <t>Excedió el tiempo de espera.</t>
         </is>
       </c>
       <c r="O28" t="n">
@@ -2512,7 +2512,7 @@
         <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R28" t="n">
         <v>1</v>
@@ -2586,7 +2586,7 @@
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R29" t="n">
         <v>1</v>
@@ -2660,7 +2660,7 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R30" t="n">
         <v>1</v>
@@ -2734,7 +2734,7 @@
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R31" t="n">
         <v>1</v>
@@ -2812,7 +2812,7 @@
         <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R32" t="n">
         <v>1</v>
@@ -2886,7 +2886,7 @@
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R33" t="n">
         <v>1</v>
@@ -2960,7 +2960,7 @@
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R34" t="n">
         <v>1</v>
@@ -3034,7 +3034,7 @@
         <v>1</v>
       </c>
       <c r="Q35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R35" t="n">
         <v>1</v>
@@ -3108,7 +3108,7 @@
         <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R36" t="n">
         <v>1</v>
@@ -3182,7 +3182,7 @@
         <v>1</v>
       </c>
       <c r="Q37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R37" t="n">
         <v>1</v>
@@ -3256,7 +3256,7 @@
         <v>1</v>
       </c>
       <c r="Q38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R38" t="n">
         <v>1</v>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>CALLATA PUMA LUCIA VERÓNICA</t>
+          <t>CALLATA PUMA LUCIA VERONICA</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3330,7 +3330,7 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R39" t="n">
         <v>1</v>
@@ -3370,7 +3370,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>CALLATA PUMA LUCIA VERÓNICA</t>
+          <t>CALLATA PUMA LUCIA VERONICA</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3404,7 +3404,7 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R40" t="n">
         <v>1</v>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>CALLATA PUMA LUCIA VERÓNICA</t>
+          <t>CALLATA PUMA LUCIA VERONICA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3478,7 +3478,7 @@
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R41" t="n">
         <v>1</v>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>CALLATA PUMA LUCIA VERÓNICA</t>
+          <t>CALLATA PUMA LUCIA VERONICA</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3552,7 +3552,7 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R42" t="n">
         <v>1</v>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>CALLATA PUMA LUCIA VERÓNICA</t>
+          <t>CALLATA PUMA LUCIA VERONICA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3626,7 +3626,7 @@
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R43" t="n">
         <v>1</v>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>CALLATA PUMA LUCIA VERÓNICA</t>
+          <t>CALLATA PUMA LUCIA VERONICA</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3700,7 +3700,7 @@
         <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R44" t="n">
         <v>1</v>
@@ -3774,7 +3774,7 @@
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R45" t="n">
         <v>1</v>
@@ -3848,7 +3848,7 @@
         <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R46" t="n">
         <v>1</v>
@@ -3922,7 +3922,7 @@
         <v>1</v>
       </c>
       <c r="Q47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R47" t="n">
         <v>1</v>
@@ -3996,7 +3996,7 @@
         <v>1</v>
       </c>
       <c r="Q48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R48" t="n">
         <v>1</v>
@@ -4070,7 +4070,7 @@
         <v>1</v>
       </c>
       <c r="Q49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R49" t="n">
         <v>1</v>
@@ -4144,7 +4144,7 @@
         <v>1</v>
       </c>
       <c r="Q50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R50" t="n">
         <v>1</v>
@@ -4218,7 +4218,7 @@
         <v>1</v>
       </c>
       <c r="Q51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R51" t="n">
         <v>1</v>
@@ -4292,7 +4292,7 @@
         <v>1</v>
       </c>
       <c r="Q52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R52" t="n">
         <v>1</v>
@@ -4366,7 +4366,7 @@
         <v>1</v>
       </c>
       <c r="Q53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R53" t="n">
         <v>1</v>
@@ -4440,7 +4440,7 @@
         <v>1</v>
       </c>
       <c r="Q54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R54" t="n">
         <v>1</v>
@@ -4512,7 +4512,7 @@
         <v>1</v>
       </c>
       <c r="Q55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R55" t="n">
         <v>1</v>
@@ -4584,7 +4584,7 @@
         <v>1</v>
       </c>
       <c r="Q56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R56" t="n">
         <v>1</v>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Excedió el tiempo de espera.</t>
+          <t>La Factura Electrónica EB01-4 no existe en los registros de SUNAT.</t>
         </is>
       </c>
       <c r="O57" t="n">
@@ -4658,7 +4658,7 @@
         <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R57" t="n">
         <v>1</v>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Excedió el tiempo de espera.</t>
+          <t>La Factura Electrónica EB01-4 no existe en los registros de SUNAT.</t>
         </is>
       </c>
       <c r="O58" t="n">
@@ -4732,7 +4732,7 @@
         <v>1</v>
       </c>
       <c r="Q58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R58" t="n">
         <v>1</v>
@@ -4806,7 +4806,7 @@
         <v>1</v>
       </c>
       <c r="Q59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R59" t="n">
         <v>1</v>
@@ -4880,7 +4880,7 @@
         <v>1</v>
       </c>
       <c r="Q60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R60" t="n">
         <v>1</v>
@@ -4954,7 +4954,7 @@
         <v>1</v>
       </c>
       <c r="Q61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R61" t="n">
         <v>1</v>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>EMPRESA DE TRANSPORTE ARENAS TOURS SRL</t>
+          <t>EMPRESA DE TRANSPORTES ARENAS TOURS S.R.L.</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>Excedió el tiempo de espera.</t>
+          <t>La Boleta de Venta Electrónica BQQ1-000129 no existe en los registros de SUNAT.</t>
         </is>
       </c>
       <c r="O62" t="n">
@@ -5028,7 +5028,7 @@
         <v>1</v>
       </c>
       <c r="Q62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R62" t="n">
         <v>1</v>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>EMPRESA DE TRANSPORTE ARENAS TOURS SRL</t>
+          <t>EMPRESA DE TRANSPORTES ARENAS TOURS S.R.L.</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Excedió el tiempo de espera.</t>
+          <t>La Boleta de Venta Electrónica BQQ1-000130 no existe en los registros de SUNAT.</t>
         </is>
       </c>
       <c r="O63" t="n">
@@ -5102,7 +5102,7 @@
         <v>1</v>
       </c>
       <c r="Q63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R63" t="n">
         <v>1</v>
@@ -5142,7 +5142,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>ALESSON CENTER EMPRESA INDIVIDUAL DE RESPONSBILIDAD LIMITADA</t>
+          <t>ALESSON CENTER EMPRESA INDIVIDUAL DE RESPONSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5176,7 +5176,7 @@
         <v>1</v>
       </c>
       <c r="Q64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R64" t="n">
         <v>1</v>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>ALESSON CENTER EMPRESA INDIVIDUAL DE RESPONSBILIDAD LIMITADA</t>
+          <t>ALESSON CENTER EMPRESA INDIVIDUAL DE RESPONSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5254,7 +5254,7 @@
         <v>1</v>
       </c>
       <c r="Q65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R65" t="n">
         <v>1</v>
@@ -5328,7 +5328,7 @@
         <v>1</v>
       </c>
       <c r="Q66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R66" t="n">
         <v>1</v>
@@ -5402,7 +5402,7 @@
         <v>1</v>
       </c>
       <c r="Q67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R67" t="n">
         <v>1</v>
@@ -5476,7 +5476,7 @@
         <v>1</v>
       </c>
       <c r="Q68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R68" t="n">
         <v>1</v>
@@ -5550,7 +5550,7 @@
         <v>1</v>
       </c>
       <c r="Q69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R69" t="n">
         <v>1</v>
@@ -5624,7 +5624,7 @@
         <v>1</v>
       </c>
       <c r="Q70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R70" t="n">
         <v>1</v>
@@ -5698,7 +5698,7 @@
         <v>1</v>
       </c>
       <c r="Q71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R71" t="n">
         <v>1</v>
@@ -5772,7 +5772,7 @@
         <v>1</v>
       </c>
       <c r="Q72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R72" t="n">
         <v>1</v>
@@ -5846,7 +5846,7 @@
         <v>1</v>
       </c>
       <c r="Q73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R73" t="n">
         <v>1</v>
@@ -5920,7 +5920,7 @@
         <v>1</v>
       </c>
       <c r="Q74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R74" t="n">
         <v>1</v>
@@ -5994,7 +5994,7 @@
         <v>1</v>
       </c>
       <c r="Q75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R75" t="n">
         <v>1</v>
@@ -6068,7 +6068,7 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R76" t="n">
         <v>1</v>
@@ -6142,7 +6142,7 @@
         <v>1</v>
       </c>
       <c r="Q77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R77" t="n">
         <v>1</v>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>A &amp; C PERU GOURMET E.I.R.L.</t>
+          <t>A &amp; C PERU GOURMET EMPRESA INDIVIDUAL DE RESPONSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -6216,7 +6216,7 @@
         <v>1</v>
       </c>
       <c r="Q78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R78" t="n">
         <v>1</v>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>A &amp; C PERU GOURMET E.I.R.L.</t>
+          <t>A &amp; C PERU GOURMET EMPRESA INDIVIDUAL DE RESPONSABILIDAD LIMITADA</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -6290,7 +6290,7 @@
         <v>1</v>
       </c>
       <c r="Q79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R79" t="n">
         <v>1</v>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>RB CHACHANI S. A. C.</t>
+          <t>RB CHACHANI S.A.C.</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -6368,7 +6368,7 @@
         <v>1</v>
       </c>
       <c r="Q80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R80" t="n">
         <v>1</v>
@@ -6442,7 +6442,7 @@
         <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R81" t="n">
         <v>1</v>
@@ -6516,7 +6516,7 @@
         <v>1</v>
       </c>
       <c r="Q82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R82" t="n">
         <v>1</v>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>INVERSIONES GENERALES KUSAQ E.I.R.L.</t>
+          <t>INVERSIONES GENERALES KUSAQ E.I.R.L. - IGK E.I.R.L.</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -6590,7 +6590,7 @@
         <v>1</v>
       </c>
       <c r="Q83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R83" t="n">
         <v>1</v>
@@ -6630,7 +6630,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>INVERSIONES GENERALES KUSAQ E.I.R.L.</t>
+          <t>INVERSIONES GENERALES KUSAQ E.I.R.L. - IGK E.I.R.L.</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -6664,7 +6664,7 @@
         <v>1</v>
       </c>
       <c r="Q84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R84" t="n">
         <v>1</v>
@@ -6704,7 +6704,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>COMPAÑÍA FOOD RETAIL S. A. C.</t>
+          <t>COMPAÑIA FOOD RETAIL S.A.C.</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -6738,7 +6738,7 @@
         <v>1</v>
       </c>
       <c r="Q85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R85" t="n">
         <v>1</v>
@@ -6778,7 +6778,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>COMPAÑÍA FOOD RETAIL S. A. C.</t>
+          <t>COMPAÑIA FOOD RETAIL S.A.C.</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -6812,7 +6812,7 @@
         <v>1</v>
       </c>
       <c r="Q86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R86" t="n">
         <v>1</v>
@@ -6852,7 +6852,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>COMPAÑÍA FOOD RETAIL S. A. C.</t>
+          <t>COMPAÑIA FOOD RETAIL S.A.C.</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6886,7 +6886,7 @@
         <v>1</v>
       </c>
       <c r="Q87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R87" t="n">
         <v>1</v>
@@ -6926,7 +6926,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>COMPAÑÍA FOOD RETAIL S. A. C.</t>
+          <t>COMPAÑIA FOOD RETAIL S.A.C.</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6960,7 +6960,7 @@
         <v>1</v>
       </c>
       <c r="Q88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R88" t="n">
         <v>1</v>
@@ -7000,7 +7000,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>COMPAÑÍA FOOD RETAIL S. A. C.</t>
+          <t>COMPAÑIA FOOD RETAIL S.A.C.</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -7034,7 +7034,7 @@
         <v>1</v>
       </c>
       <c r="Q89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R89" t="n">
         <v>1</v>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>EMPRESA DE SERVICIOS MULTIPLES CESAR VALLEJO AIRPORT S. A.</t>
+          <t>EMPRESA DE SERVICIOS MULTIPLES CESAR VALLEJO AIRPORT S.A.</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -7108,7 +7108,7 @@
         <v>1</v>
       </c>
       <c r="Q90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R90" t="n">
         <v>1</v>
@@ -7182,7 +7182,7 @@
         <v>1</v>
       </c>
       <c r="Q91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R91" t="n">
         <v>1</v>
@@ -7256,7 +7256,7 @@
         <v>1</v>
       </c>
       <c r="Q92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R92" t="n">
         <v>1</v>
@@ -7330,7 +7330,7 @@
         <v>1</v>
       </c>
       <c r="Q93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R93" t="n">
         <v>1</v>
@@ -7404,7 +7404,7 @@
         <v>1</v>
       </c>
       <c r="Q94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R94" t="n">
         <v>1</v>
@@ -7444,7 +7444,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E. I .R. L.</t>
+          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E.I.R.L.</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -7478,7 +7478,7 @@
         <v>1</v>
       </c>
       <c r="Q95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R95" t="n">
         <v>1</v>
@@ -7518,7 +7518,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E. I .R. L.</t>
+          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E.I.R.L.</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -7552,7 +7552,7 @@
         <v>1</v>
       </c>
       <c r="Q96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R96" t="n">
         <v>1</v>
@@ -7592,7 +7592,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E. I .R. L.</t>
+          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E.I.R.L.</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -7626,7 +7626,7 @@
         <v>1</v>
       </c>
       <c r="Q97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R97" t="n">
         <v>1</v>
@@ -7666,7 +7666,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E. I .R. L.</t>
+          <t>DISTRIBUCIONES Y NEGOCIOS JEFFERSON E.I.R.L.</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -7700,7 +7700,7 @@
         <v>1</v>
       </c>
       <c r="Q98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R98" t="n">
         <v>1</v>

</xml_diff>